<commit_message>
corrigindo leitura de planilha
</commit_message>
<xml_diff>
--- a/InputModelo.xlsx
+++ b/InputModelo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geovane.carvalho\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geovane.carvalho\Desktop\Extensão\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A1FD4F-A982-42C2-84D9-10FB6EDCDBFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4C1AF6-183C-45A5-A2E6-18942901B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15816" xr2:uid="{192CF486-777D-4261-B871-567073522E09}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{192CF486-777D-4261-B871-567073522E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -37,23 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
-  <si>
-    <t>Misc.TBRA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
   <si>
     <t>1/1</t>
   </si>
   <si>
-    <t>0380-9200-0</t>
-  </si>
-  <si>
-    <t>0452-0120-3</t>
-  </si>
-  <si>
-    <t>0460-0084-4</t>
-  </si>
-  <si>
     <t>Site A</t>
   </si>
   <si>
@@ -90,20 +78,38 @@
     <t>LOCAL EXECUCAO OBRA</t>
   </si>
   <si>
-    <t>Miscelânea</t>
+    <t>PB CLASSE LFO</t>
+  </si>
+  <si>
+    <t>PB CLASSE P</t>
+  </si>
+  <si>
+    <t>PB CLASSE L</t>
+  </si>
+  <si>
+    <t>PB CLASSE C</t>
+  </si>
+  <si>
+    <t>Estação HGA</t>
+  </si>
+  <si>
+    <t>PB CLASSE CFO</t>
+  </si>
+  <si>
+    <t>PB CLASSE BFO</t>
+  </si>
+  <si>
+    <t>PB CLASSE G</t>
   </si>
   <si>
     <t>PB CLASSE LE</t>
-  </si>
-  <si>
-    <t>PB CLASSE LFO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,12 +126,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF383D41"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF212529"/>
@@ -134,14 +134,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF383D41"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -167,34 +168,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -202,6 +185,18 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +398,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -457,8 +452,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}" name="Tabela1" displayName="Tabela1" ref="A1:J8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J8" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}" name="Tabela1" displayName="Tabela1" ref="A1:J12" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J12" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{F4EB1EE5-BE24-4BD4-9B71-305E989170F6}" name="ID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{4B241DE7-21A2-41A9-8815-D9DF45ED195D}" name="PRANCHA" dataDxfId="8"/>
@@ -772,7 +767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{100581EE-D5FB-4D36-A2CF-C29070646DE3}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -788,207 +783,249 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="F1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="G1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="H1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="I1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="J1" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>592256</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="5">
-        <v>888888</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5">
-        <v>1000</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="C2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="8">
+        <v>100021</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="6">
+        <v>28.33</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>592256</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="8">
+        <v>221708</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="6">
         <v>1</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="5">
-        <v>888888</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5">
-        <v>50</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>592256</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="5">
-        <v>888888</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="C4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="8">
+        <v>226041</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="6">
+        <v>2</v>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5">
-        <v>2</v>
-      </c>
-      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="9">
+      <c r="A5" s="1">
         <v>592256</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>1</v>
+      <c r="B5" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="1">
-        <v>520985</v>
-      </c>
-      <c r="F5" s="11">
-        <v>1</v>
+        <v>240079</v>
+      </c>
+      <c r="F5" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="9">
+      <c r="A6" s="1">
         <v>592256</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>1</v>
+      <c r="B6" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1">
-        <v>290107</v>
-      </c>
-      <c r="F6" s="11">
-        <v>50</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>6</v>
+        <v>290689</v>
+      </c>
+      <c r="F6" s="5">
+        <v>288</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="9">
+      <c r="A7" s="1">
         <v>592256</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>1</v>
+      <c r="B7" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="1">
+        <v>293105</v>
+      </c>
+      <c r="F7" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>592256</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="1">
+        <v>420018</v>
+      </c>
+      <c r="F8" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>592256</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1">
+        <v>460036</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>592256</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1">
+        <v>520985</v>
+      </c>
+      <c r="F10" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>592256</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="1">
         <v>290107</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F11" s="5">
+        <v>50</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>592256</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="1">
+        <v>290107</v>
+      </c>
+      <c r="F12" s="5">
         <v>1000</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
-        <v>592256</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="J12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5">
-        <v>888888</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5">
-        <v>24</v>
-      </c>
-      <c r="J8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
ajuste de mapeamento de campo com csv
</commit_message>
<xml_diff>
--- a/InputModelo.xlsx
+++ b/InputModelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geovane.carvalho\Desktop\Extensão\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4C1AF6-183C-45A5-A2E6-18942901B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB6CDC1-0393-4329-A3E7-E272EE615A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{192CF486-777D-4261-B871-567073522E09}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>1/1</t>
   </si>
@@ -78,7 +78,13 @@
     <t>LOCAL EXECUCAO OBRA</t>
   </si>
   <si>
-    <t>PB CLASSE LFO</t>
+    <t>Misc.TBRA</t>
+  </si>
+  <si>
+    <t>0452-0120-3</t>
+  </si>
+  <si>
+    <t>0460-0084-4</t>
   </si>
   <si>
     <t>PB CLASSE P</t>
@@ -87,29 +93,14 @@
     <t>PB CLASSE L</t>
   </si>
   <si>
-    <t>PB CLASSE C</t>
-  </si>
-  <si>
-    <t>Estação HGA</t>
-  </si>
-  <si>
-    <t>PB CLASSE CFO</t>
-  </si>
-  <si>
-    <t>PB CLASSE BFO</t>
-  </si>
-  <si>
-    <t>PB CLASSE G</t>
-  </si>
-  <si>
-    <t>PB CLASSE LE</t>
+    <t>0380-9200-0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,14 +130,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -168,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -185,18 +168,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,8 +423,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}" name="Tabela1" displayName="Tabela1" ref="A1:J12" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J12" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}" name="Tabela1" displayName="Tabela1" ref="A1:J7" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J7" xr:uid="{2F312025-B7BE-4F9F-B05A-7C298157D64C}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{F4EB1EE5-BE24-4BD4-9B71-305E989170F6}" name="ID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{4B241DE7-21A2-41A9-8815-D9DF45ED195D}" name="PRANCHA" dataDxfId="8"/>
@@ -767,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{100581EE-D5FB-4D36-A2CF-C29070646DE3}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -815,71 +786,58 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="1">
         <v>592256</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="8">
+      <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="1">
         <v>100021</v>
       </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="6">
+      <c r="F2" s="5">
         <v>28.33</v>
       </c>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="8">
+      <c r="A3" s="1">
         <v>592256</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="8">
+      <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="1">
         <v>221708</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>1</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="8"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
+      <c r="A4" s="1">
         <v>592256</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="8">
-        <v>226041</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="6">
-        <v>2</v>
-      </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="8" t="s">
-        <v>17</v>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1">
+        <v>888888</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="1">
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -890,13 +848,20 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1">
-        <v>240079</v>
-      </c>
-      <c r="F5" s="5">
-        <v>2</v>
+        <v>888888</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -907,13 +872,20 @@
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1">
-        <v>290689</v>
-      </c>
-      <c r="F6" s="5">
-        <v>288</v>
+        <v>888888</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="1">
+        <v>50</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -924,104 +896,17 @@
         <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1">
-        <v>293105</v>
-      </c>
-      <c r="F7" s="5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>592256</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="1">
-        <v>420018</v>
-      </c>
-      <c r="F8" s="5">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>592256</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="1">
-        <v>460036</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0.28000000000000003</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>592256</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1">
-        <v>520985</v>
-      </c>
-      <c r="F10" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>592256</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1">
-        <v>290107</v>
-      </c>
-      <c r="F11" s="5">
-        <v>50</v>
-      </c>
-      <c r="J11" s="1" t="s">
+        <v>888888</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="1">
         <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>592256</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1">
-        <v>290107</v>
-      </c>
-      <c r="F12" s="5">
-        <v>1000</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>